<commit_message>
Big update: v6 tracker, v5 gantt
comprehensive update to the hub to reflect the progress up to Week 10 - v5 gantt and v6 tracker now available on 04 Oct
</commit_message>
<xml_diff>
--- a/files/Archive/Spinney_Budget_Tracker_v5.xlsx
+++ b/files/Archive/Spinney_Budget_Tracker_v5.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="383">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="402">
   <si>
     <t xml:space="preserve">Spinney External Works — Budget Summary</t>
   </si>
@@ -143,7 +143,7 @@
     <t xml:space="preserve">Snapshot</t>
   </si>
   <si>
-    <t xml:space="preserve">Week 9 — overall, still on plan. Roofline works (£2,100) is a genuine new addition, own scope and own budget. Chimney and coping remain fully complete and settled (Gate 1 cleared 18 Aug). Decking is the active workstream: substructure re-planned to ~22 Sep across both sides plus the new shed area, board-laying to follow once Gates 2 and 3 clear. Materials pool is back under cap. Contingency has six genuine draws but is still comfortably under half-drawn. Nothing here suggests a budget problem.</t>
+    <t xml:space="preserve">Week 9 — overall, still on plan, though 11 Sep was a big day for Contingency: £2,115 in extra decking/shed digging and fence repositioning (side a), taking Contingency to £2,737.64 drawn of £5,000 — still under, but the pot has moved significantly. Rubbish removal pool is now £100 over its £1,360 cap after the wood removal correction. Chimney and coping remain fully complete and settled. Decking substructure continues toward the ~22 Sep target. Nothing here is a crisis, but Contingency is worth watching now it is over half-drawn.</t>
   </si>
   <si>
     <t xml:space="preserve">• Chimney</t>
@@ -251,7 +251,7 @@
     <t xml:space="preserve">Rubbish removal (pooled, all 3 workstreams)</t>
   </si>
   <si>
-    <t xml:space="preserve">Decking's £1,200 share largely untested — see snapshot caveat</t>
+    <t xml:space="preserve">£100 OVER the £1,360 cap — the wood removal correction (£350 est. → £680 actual, charged per trip) pushed it over. Flagged, not hidden; cap left as-is per the same approach used for Materials pooled.</t>
   </si>
   <si>
     <t xml:space="preserve">Roofline works (new, 4 Sep estimate)</t>
@@ -260,7 +260,7 @@
     <t xml:space="preserve">New scope, own budget — gutters, fascia/soffit, slates, barge boards. £40 rubbish removal reclassified to the pooled Rubbish removal fund. Not yet started or invoiced; quote used as placeholder actual until real costs land.</t>
   </si>
   <si>
-    <t xml:space="preserve">£622.64 drawn of the £5,000 pot (condensation-prep £276.42 + chimney cowl £62.90 + V4 screw top-ups £283.32) — £4,377.36 remaining. Variance here just means 'not yet drawn', not a saving.</t>
+    <t xml:space="preserve">£2,737.64 drawn of the £5,000 pot — £2,262.36 remaining. Big jump 11 Sep: £2,115 for extra decking/shed digging and fence repositioning (side a), on top of the earlier six smaller draws (condensation-prep, cowl, two screw top-ups).</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL (as spent/committed to date)</t>
@@ -725,16 +725,13 @@
     <t xml:space="preserve">TBC (cash)</t>
   </si>
   <si>
-    <t xml:space="preserve">Old decking substructure wood collection — £350 cash, collection expected this week</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cash (pending)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not yet collected/paid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8 Sep: confirmed price for collecting the old decking substructure wood. Not a skip — separate wood-collection charge, same pooled fund since it's decking-related waste removal.</t>
+    <t xml:space="preserve">Old decking substructure wood collection — PAID 11 Sep, £680 cash (was estimated £350; charged per trip, 2 trips)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Original £350 estimate corrected 11 Sep — supplier charges per trip, and 2 trips were needed for this volume of wood. Same job, not a separate charge. From the decking quote scope, so pooled here per Ryan's confirmation.</t>
   </si>
   <si>
     <t xml:space="preserve">Labour — gutter replacement (both parapet sides + lower rear elevation), fascia/soffit extension, slate replacement, barge board trim</t>
@@ -758,6 +755,33 @@
     <t xml:space="preserve">Per estimate 4 Sep. RECLASSIFIED 8 Sep from Roofline works into the pooled Rubbish removal fund — same rationale as the other pooled items (chimney/coping/decking rubbish already share this fund).</t>
   </si>
   <si>
+    <t xml:space="preserve">Named purpose #11 — extra digging: wider deck gate area (1 day x2 people) + additional deck/shed area (1 day x2 people)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash (10% disc.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quoted £1,400, cash-discounted to £1,260. Tied to tasks 2.2 (wider gate area) + 2.6 (shed/additional deck) — mixed purpose, doesn't cleanly split between the two. Part of Luke's 11 Sep extras invoice, £2,115 total across 4 items.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Named purpose #12 — cleanup after machines (2hrs) + dig up small tree (2hrs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quoted £200, cash-discounted to £180. Tied to tasks 2.2/2.6 excavation cleanup. Small tree dig — distinct from task 3.4's external tree/bush clearing company. Part of the same 11 Sep extras invoice.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Named purpose #13 — fence move, chimney side (side a boundary reclaim from neighbour, to enable the wider decking area)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quoted £700 for 'move fence and do spurs to make a full day', but spurs (task 3.3, side b) did NOT happen — only £350 charged for the fence move itself, cash-discounted to £315. NOT the same fence as 3.3 (side b, concrete spurs) or 3.5 (TPO/tree-dependent). New task — see Gantt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Named purpose #14 — extra frame for wider deck gate area (1 person; no extra charge for boarding)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quoted £400, cash-discounted to £360. Tied to task 2.2 (decking side a widening substructure/framing).</t>
+  </si>
+  <si>
     <t xml:space="preserve">TOTAL (all lines)</t>
   </si>
   <si>
@@ -818,9 +842,6 @@
     <t xml:space="preserve">PREPAYMENT vs chimney phase-start invoice: pay £1,528.29 of the £1,640 when it lands</t>
   </si>
   <si>
-    <t xml:space="preserve">Cash</t>
-  </si>
-  <si>
     <t xml:space="preserve">Scaffold erection payment — chimney share (pro-rata of £2,000 cash)</t>
   </si>
   <si>
@@ -1034,6 +1055,39 @@
     <t xml:space="preserve">Invoice received and paid 10 Sep, delivery scheduled 11 Sep. Amount inferred from purpose #8's confirmed rate — no invoice number/exact figure given; flag if actual differs.</t>
   </si>
   <si>
+    <t xml:space="preserve">N/A (cash)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Old decking substructure wood collection — corrected to £680 (was £350 est.), charged per trip, 2 trips</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same job as the earlier £350 estimate — supplier charges per trip, not a flat rate. Not a separate/additional charge.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extra digging — wider gate area + shed/additional deck (named purpose #11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quoted £1,400, 10% cash discount applied. Part of Luke's 11 Sep extras, £2,115 total across 4 items.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cleanup after machines + dig up small tree (named purpose #12)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quoted £200, 10% cash discount applied.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fence move, chimney side/side a boundary reclaim (named purpose #13)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quoted £700 for move+spurs, but spurs (3.3, side b) didn't happen — only £350 charged, 10% cash discount applied.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extra frame, wider deck gate area (named purpose #14)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quoted £400, 10% cash discount applied.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Skip Hire Log — pooled rubbish-removal drawdown</t>
   </si>
   <si>
@@ -1082,10 +1136,7 @@
     <t xml:space="preserve">8 cubic yard, exchange — collects filled skip, delivers empty (INV-11375, ref 26030)</t>
   </si>
   <si>
-    <t xml:space="preserve">TBC (cash collection)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Old decking substructure wood collection — £350 cash, pending, expected this week</t>
+    <t xml:space="preserve">Old decking substructure wood collection — PAID 11 Sep, £680 cash (was estimated £350; supplier charges per trip, 2 trips required)</t>
   </si>
   <si>
     <t xml:space="preserve">Decking substructure, both sides</t>
@@ -1145,7 +1196,7 @@
     <t xml:space="preserve">Contingency Drawdown — £5,000 pot (agreed Lara/Luke, 1 Jul 2026)</t>
   </si>
   <si>
-    <t xml:space="preserve">Named purposes: fence move/repair labour · ~~soakaway fix before decking~~ CANCELLED 1 Sep, cost-benefit not worth it, nothing drawn · drainage by the garage · additional curved-decking labour · cement &amp; bricks · coping condensation-prep (£276.42, purpose #6) · chimney cowl upgrade (£62.90, purpose #7) · V4 screw top-up (£141.66, purpose #8) · V4 screw top-up #2 (£141.66, purpose #9, PAID 10 Sep, delivery 11 Sep) · digger + barrow loader hire (est. £530, purpose #10, on hire until 10 Sep, mixed purpose — side (a) decking widening + new shed excavation). Luke's labour from this pot invoiced at 10% discount (extended 20 Jul) — condensation-prep, the cowl, and both screw top-ups were/are bank transfer/direct paid, not cash, so no discount applies to any of them. Curved-decking extra labour discount status TBC. Pipe investigation (task 2.2) RESOLVED 4 Sep: no leaking pipe found.</t>
+    <t xml:space="preserve">Named purposes: ~~fence move/repair labour~~ SUPERSEDED — see purpose #13 · ~~soakaway fix before decking~~ CANCELLED 1 Sep, cost-benefit not worth it, nothing drawn · drainage by the garage · additional curved-decking labour · cement &amp; bricks · coping condensation-prep (£276.42, purpose #6) · chimney cowl upgrade (£62.90, purpose #7) · V4 screw top-up (£141.66, purpose #8) · V4 screw top-up #2 (£141.66, purpose #9, PAID 10 Sep) · digger + barrow loader hire (est. £530, purpose #10, mixed purpose — side (a) decking widening + new shed excavation) · extra digging, wider gate area + shed/additional deck (£1,260, purpose #11, PAID 11 Sep) · cleanup + small tree dig (£180, purpose #12, PAID 11 Sep) · fence move, chimney side/side a boundary reclaim (£315, purpose #13, PAID 11 Sep — this is the original 'fence move/repair labour' purpose, now specific) · extra frame, wider deck gate area (£360, purpose #14, PAID 11 Sep). Purposes #11-14 are all part of Luke's 11 Sep extras invoice (£2,350 quoted, £2,115 paid after 10% cash discount) — covers extra decking/shed digging and fence repositioning, side a, needed before any decking boards go down. Luke's labour from this pot: condensation-prep, the cowl, and both screw top-ups were bank transfer/direct paid (no discount); the 11 Sep extras were cash (10% discount applied). Curved-decking extra labour discount status TBC. Pipe investigation (task 2.2) RESOLVED 4 Sep: no leaking pipe found.</t>
   </si>
   <si>
     <t xml:space="preserve">Opening pot:</t>
@@ -1176,6 +1227,12 @@
   </si>
   <si>
     <t xml:space="preserve">V4 screw top-up #2 (named purpose #9) — PAID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cleanup + small tree dig (named purpose #12)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fence move, chimney side/side a boundary (named purpose #13)</t>
   </si>
 </sst>
 </file>
@@ -1192,7 +1249,7 @@
     <numFmt numFmtId="170" formatCode="General"/>
     <numFmt numFmtId="171" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1310,6 +1367,14 @@
     </font>
     <font>
       <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FFDC2626"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="13"/>
       <color rgb="FF0F766E"/>
       <name val="Calibri"/>
@@ -1439,303 +1504,303 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="16" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="16" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1752,7 +1817,7 @@
     <indexedColors>
       <rgbColor rgb="FF000000"/>
       <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FFDC2626"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -2104,15 +2169,15 @@
       </c>
       <c r="D7" s="10" t="n">
         <f aca="false">SUMIF('Invoice Register'!$B:$B,$A7,'Invoice Register'!$F:$F)</f>
-        <v>622.64</v>
+        <v>2737.64</v>
       </c>
       <c r="E7" s="10" t="n">
         <f aca="false">SUMIFS('Invoice Register'!$F:$F,'Invoice Register'!$B:$B,$A7,'Invoice Register'!$G:$G,"&lt;&gt;")</f>
-        <v>622.64</v>
+        <v>2737.64</v>
       </c>
       <c r="F7" s="10" t="n">
         <f aca="false">C7-D7</f>
-        <v>4377.36</v>
+        <v>2262.36</v>
       </c>
       <c r="G7" s="11" t="s">
         <v>18</v>
@@ -2208,15 +2273,15 @@
       </c>
       <c r="D11" s="16" t="n">
         <f aca="false">SUMIF('Invoice Register'!$B:$B,$A11,'Invoice Register'!$F:$F)</f>
-        <v>780</v>
+        <v>1460</v>
       </c>
       <c r="E11" s="16" t="n">
         <f aca="false">SUMIFS('Invoice Register'!$F:$F,'Invoice Register'!$B:$B,$A11,'Invoice Register'!$G:$G,"&lt;&gt;")</f>
-        <v>780</v>
+        <v>1460</v>
       </c>
       <c r="F11" s="16" t="n">
         <f aca="false">C11-D11</f>
-        <v>580</v>
+        <v>-100</v>
       </c>
       <c r="G11" s="17" t="s">
         <v>28</v>
@@ -2259,15 +2324,15 @@
       </c>
       <c r="D13" s="15" t="n">
         <f aca="false">D5+D6+D7</f>
-        <v>39251.63</v>
+        <v>41366.63</v>
       </c>
       <c r="E13" s="15" t="n">
         <f aca="false">E5+E6+E7</f>
-        <v>39251.63</v>
+        <v>41366.63</v>
       </c>
       <c r="F13" s="15" t="n">
         <f aca="false">F5+F6+F7</f>
-        <v>15577.36</v>
+        <v>13462.36</v>
       </c>
       <c r="G13" s="22"/>
     </row>
@@ -2305,15 +2370,15 @@
       </c>
       <c r="D15" s="28" t="n">
         <f aca="false">D11+D12+D13</f>
-        <v>40031.63</v>
+        <v>42826.63</v>
       </c>
       <c r="E15" s="28" t="n">
         <f aca="false">E11+E12+E13</f>
-        <v>40031.63</v>
+        <v>42826.63</v>
       </c>
       <c r="F15" s="28" t="n">
         <f aca="false">F11+F12+F13</f>
-        <v>18257.36</v>
+        <v>15462.36</v>
       </c>
       <c r="G15" s="27"/>
     </row>
@@ -2323,7 +2388,7 @@
       </c>
       <c r="B16" s="29" t="n">
         <f aca="false">'Contingency Drawdown'!$D$4</f>
-        <v>4377.36</v>
+        <v>2262.36</v>
       </c>
     </row>
   </sheetData>
@@ -2596,10 +2661,10 @@
         <v>1360</v>
       </c>
       <c r="C24" s="42" t="n">
-        <v>780</v>
+        <v>1460</v>
       </c>
       <c r="D24" s="43" t="n">
-        <v>-580</v>
+        <v>100</v>
       </c>
       <c r="E24" s="14" t="s">
         <v>74</v>
@@ -2630,10 +2695,10 @@
         <v>5000</v>
       </c>
       <c r="C26" s="36" t="n">
-        <v>622.64</v>
+        <v>2737.64</v>
       </c>
       <c r="D26" s="41" t="n">
-        <v>-4377.36</v>
+        <v>-2262.36</v>
       </c>
       <c r="E26" s="8" t="s">
         <v>77</v>
@@ -2647,10 +2712,10 @@
         <v>69618.99</v>
       </c>
       <c r="C27" s="1" t="n">
-        <v>53262.32</v>
+        <v>56057.32</v>
       </c>
       <c r="D27" s="45" t="n">
-        <v>-16356.67</v>
+        <v>-13561.67</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3254,7 +3319,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
@@ -4067,16 +4132,16 @@
       <c r="D34" s="54"/>
       <c r="E34" s="54"/>
       <c r="F34" s="54" t="n">
-        <v>350</v>
+        <v>680</v>
       </c>
       <c r="G34" s="54" t="s">
         <v>233</v>
       </c>
       <c r="H34" s="54" t="s">
+        <v>102</v>
+      </c>
+      <c r="I34" s="8" t="s">
         <v>234</v>
-      </c>
-      <c r="I34" s="8" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4087,7 +4152,7 @@
         <v>14</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D35" s="54"/>
       <c r="E35" s="54"/>
@@ -4101,7 +4166,7 @@
         <v>203</v>
       </c>
       <c r="I35" s="20" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4112,7 +4177,7 @@
         <v>14</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="D36" s="54"/>
       <c r="E36" s="54"/>
@@ -4126,7 +4191,7 @@
         <v>170</v>
       </c>
       <c r="I36" s="20" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4137,7 +4202,7 @@
         <v>14</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="D37" s="54"/>
       <c r="E37" s="54"/>
@@ -4151,7 +4216,7 @@
         <v>170</v>
       </c>
       <c r="I37" s="20" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4162,7 +4227,7 @@
         <v>14</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D38" s="54"/>
       <c r="E38" s="54"/>
@@ -4176,16 +4241,116 @@
         <v>170</v>
       </c>
       <c r="I38" s="20" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="54" t="s">
+        <v>16</v>
+      </c>
+      <c r="B39" s="54" t="s">
+        <v>14</v>
+      </c>
+      <c r="C39" s="8" t="s">
         <v>242</v>
       </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C39" s="63" t="s">
+      <c r="D39" s="54"/>
+      <c r="E39" s="54"/>
+      <c r="F39" s="58" t="n">
+        <v>1260</v>
+      </c>
+      <c r="G39" s="54" t="s">
         <v>243</v>
       </c>
-      <c r="F39" s="64" t="n">
-        <f aca="false">SUM(F5:F38)</f>
-        <v>70066.47</v>
+      <c r="H39" s="54" t="s">
+        <v>102</v>
+      </c>
+      <c r="I39" s="8" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="54" t="s">
+        <v>16</v>
+      </c>
+      <c r="B40" s="54" t="s">
+        <v>14</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="D40" s="54"/>
+      <c r="E40" s="54"/>
+      <c r="F40" s="58" t="n">
+        <v>180</v>
+      </c>
+      <c r="G40" s="54" t="s">
+        <v>243</v>
+      </c>
+      <c r="H40" s="54" t="s">
+        <v>102</v>
+      </c>
+      <c r="I40" s="8" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="81.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="54" t="s">
+        <v>16</v>
+      </c>
+      <c r="B41" s="54" t="s">
+        <v>14</v>
+      </c>
+      <c r="C41" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="D41" s="54"/>
+      <c r="E41" s="54"/>
+      <c r="F41" s="58" t="n">
+        <v>315</v>
+      </c>
+      <c r="G41" s="54" t="s">
+        <v>243</v>
+      </c>
+      <c r="H41" s="54" t="s">
+        <v>102</v>
+      </c>
+      <c r="I41" s="8" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="54" t="s">
+        <v>16</v>
+      </c>
+      <c r="B42" s="54" t="s">
+        <v>14</v>
+      </c>
+      <c r="C42" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="D42" s="54"/>
+      <c r="E42" s="54"/>
+      <c r="F42" s="58" t="n">
+        <v>360</v>
+      </c>
+      <c r="G42" s="54" t="s">
+        <v>243</v>
+      </c>
+      <c r="H42" s="54" t="s">
+        <v>102</v>
+      </c>
+      <c r="I42" s="8" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C43" s="63" t="s">
+        <v>251</v>
+      </c>
+      <c r="F43" s="64" t="n">
+        <f aca="false">SUM(F5:F42)</f>
+        <v>72511.47</v>
       </c>
     </row>
   </sheetData>
@@ -4204,7 +4369,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13"/>
@@ -4218,17 +4383,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>3</v>
@@ -4237,19 +4402,19 @@
         <v>4</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>9</v>
@@ -4266,10 +4431,10 @@
         <v>11</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="F5" s="18" t="n">
         <v>32228.99</v>
@@ -4278,10 +4443,10 @@
         <v>46212</v>
       </c>
       <c r="H5" s="54" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4292,13 +4457,13 @@
         <v>23</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
       <c r="F6" s="18" t="n">
         <v>311.98</v>
@@ -4307,10 +4472,10 @@
         <v>46223</v>
       </c>
       <c r="H6" s="54" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4321,13 +4486,13 @@
         <v>19</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="F7" s="18" t="n">
         <v>111.71</v>
@@ -4336,10 +4501,10 @@
         <v>46223</v>
       </c>
       <c r="H7" s="54" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4353,10 +4518,10 @@
         <v>105</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>263</v>
+        <v>233</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="F8" s="18" t="n">
         <v>937.5</v>
@@ -4365,10 +4530,10 @@
         <v>46223</v>
       </c>
       <c r="H8" s="54" t="s">
-        <v>263</v>
+        <v>233</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4382,10 +4547,10 @@
         <v>14</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="F9" s="18" t="n">
         <v>3088.3</v>
@@ -4397,7 +4562,7 @@
         <v>221</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4408,13 +4573,13 @@
         <v>23</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>270</v>
+        <v>277</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>271</v>
+        <v>278</v>
       </c>
       <c r="F10" s="18" t="n">
         <v>162.96</v>
@@ -4423,10 +4588,10 @@
         <v>46225</v>
       </c>
       <c r="H10" s="54" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="I10" s="8" t="s">
-        <v>272</v>
+        <v>279</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4437,13 +4602,13 @@
         <v>23</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="F11" s="18" t="n">
         <v>148.53</v>
@@ -4452,10 +4617,10 @@
         <v>46238</v>
       </c>
       <c r="H11" s="54" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4469,10 +4634,10 @@
         <v>14</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>263</v>
+        <v>233</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="F12" s="18" t="n">
         <v>1710</v>
@@ -4481,10 +4646,10 @@
         <v>46241</v>
       </c>
       <c r="H12" s="54" t="s">
-        <v>263</v>
+        <v>233</v>
       </c>
       <c r="I12" s="8" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4498,10 +4663,10 @@
         <v>210</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="F13" s="18" t="n">
         <v>62.9</v>
@@ -4510,10 +4675,10 @@
         <v>46244</v>
       </c>
       <c r="H13" s="54" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>281</v>
+        <v>288</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4524,13 +4689,13 @@
         <v>26</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>283</v>
+        <v>290</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>284</v>
+        <v>291</v>
       </c>
       <c r="F14" s="18" t="n">
         <v>344.16</v>
@@ -4539,10 +4704,10 @@
         <v>46244</v>
       </c>
       <c r="H14" s="54" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="I14" s="8" t="s">
-        <v>285</v>
+        <v>292</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4553,13 +4718,13 @@
         <v>26</v>
       </c>
       <c r="C15" s="67" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="D15" s="67" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="E15" s="68" t="s">
-        <v>287</v>
+        <v>294</v>
       </c>
       <c r="F15" s="69" t="n">
         <v>-344.16</v>
@@ -4571,7 +4736,7 @@
         <v>17</v>
       </c>
       <c r="I15" s="68" t="s">
-        <v>288</v>
+        <v>295</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4582,13 +4747,13 @@
         <v>26</v>
       </c>
       <c r="C16" s="67" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="D16" s="67" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="E16" s="68" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="F16" s="69" t="n">
         <v>390</v>
@@ -4600,7 +4765,7 @@
         <v>203</v>
       </c>
       <c r="I16" s="68" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4611,13 +4776,13 @@
         <v>26</v>
       </c>
       <c r="C17" s="67" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="D17" s="67" t="s">
-        <v>293</v>
+        <v>300</v>
       </c>
       <c r="E17" s="68" t="s">
-        <v>294</v>
+        <v>301</v>
       </c>
       <c r="F17" s="69" t="n">
         <v>390</v>
@@ -4629,7 +4794,7 @@
         <v>203</v>
       </c>
       <c r="I17" s="68" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4643,10 +4808,10 @@
         <v>14</v>
       </c>
       <c r="D18" s="67" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="E18" s="68" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="F18" s="69" t="n">
         <v>1900</v>
@@ -4658,7 +4823,7 @@
         <v>221</v>
       </c>
       <c r="I18" s="68" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4672,10 +4837,10 @@
         <v>14</v>
       </c>
       <c r="D19" s="67" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="E19" s="68" t="s">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="F19" s="69" t="n">
         <v>250</v>
@@ -4687,7 +4852,7 @@
         <v>221</v>
       </c>
       <c r="I19" s="68" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4698,13 +4863,13 @@
         <v>23</v>
       </c>
       <c r="C20" s="67" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="D20" s="67" t="s">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="E20" s="68" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="F20" s="69" t="n">
         <v>47.99</v>
@@ -4713,10 +4878,10 @@
         <v>46250</v>
       </c>
       <c r="H20" s="67" t="s">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="I20" s="68" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4730,10 +4895,10 @@
         <v>214</v>
       </c>
       <c r="D21" s="67" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="E21" s="68" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="F21" s="69" t="n">
         <v>481.28</v>
@@ -4745,7 +4910,7 @@
         <v>221</v>
       </c>
       <c r="I21" s="68" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4756,13 +4921,13 @@
         <v>23</v>
       </c>
       <c r="C22" s="67" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="D22" s="67" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="E22" s="68" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="F22" s="69" t="n">
         <v>-72.23</v>
@@ -4774,7 +4939,7 @@
         <v>221</v>
       </c>
       <c r="I22" s="68" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4788,10 +4953,10 @@
         <v>214</v>
       </c>
       <c r="D23" s="67" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="E23" s="68" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="F23" s="69" t="n">
         <v>26.42</v>
@@ -4803,7 +4968,7 @@
         <v>221</v>
       </c>
       <c r="I23" s="68" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4817,10 +4982,10 @@
         <v>214</v>
       </c>
       <c r="D24" s="67" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="E24" s="68" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="F24" s="69" t="n">
         <v>40.18</v>
@@ -4832,7 +4997,7 @@
         <v>221</v>
       </c>
       <c r="I24" s="68" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4846,10 +5011,10 @@
         <v>14</v>
       </c>
       <c r="D25" s="67" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="E25" s="68" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
       <c r="F25" s="69" t="n">
         <v>4400</v>
@@ -4861,7 +5026,7 @@
         <v>221</v>
       </c>
       <c r="I25" s="68" t="s">
-        <v>320</v>
+        <v>327</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4875,10 +5040,10 @@
         <v>105</v>
       </c>
       <c r="D26" s="54" t="s">
-        <v>263</v>
+        <v>233</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="F26" s="54" t="n">
         <v>1062.5</v>
@@ -4887,10 +5052,10 @@
         <v>46223</v>
       </c>
       <c r="H26" s="54" t="s">
-        <v>263</v>
+        <v>233</v>
       </c>
       <c r="I26" s="8" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4907,7 +5072,7 @@
         <v>17</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="F27" s="54" t="n">
         <v>562.5</v>
@@ -4919,7 +5084,7 @@
         <v>203</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>324</v>
+        <v>331</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4936,7 +5101,7 @@
         <v>17</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="F28" s="54" t="n">
         <v>637.5</v>
@@ -4948,7 +5113,7 @@
         <v>203</v>
       </c>
       <c r="I28" s="8" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4962,10 +5127,10 @@
         <v>11</v>
       </c>
       <c r="D29" s="54" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
       <c r="F29" s="54" t="n">
         <v>141.66</v>
@@ -4977,7 +5142,7 @@
         <v>221</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="108.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4991,10 +5156,10 @@
         <v>14</v>
       </c>
       <c r="D30" s="54" t="s">
-        <v>263</v>
+        <v>233</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>330</v>
+        <v>337</v>
       </c>
       <c r="F30" s="54" t="n">
         <v>2000</v>
@@ -5003,10 +5168,10 @@
         <v>46269</v>
       </c>
       <c r="H30" s="54" t="s">
-        <v>263</v>
+        <v>233</v>
       </c>
       <c r="I30" s="8" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="81.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5020,10 +5185,10 @@
         <v>11</v>
       </c>
       <c r="D31" s="54" t="s">
-        <v>332</v>
+        <v>339</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
       <c r="F31" s="54" t="n">
         <v>141.66</v>
@@ -5035,7 +5200,152 @@
         <v>203</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>334</v>
+        <v>341</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="70" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B32" s="54" t="s">
+        <v>26</v>
+      </c>
+      <c r="C32" s="54" t="s">
+        <v>203</v>
+      </c>
+      <c r="D32" s="54" t="s">
+        <v>342</v>
+      </c>
+      <c r="E32" s="8" t="s">
+        <v>343</v>
+      </c>
+      <c r="F32" s="54" t="n">
+        <v>680</v>
+      </c>
+      <c r="G32" s="70" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H32" s="54" t="s">
+        <v>233</v>
+      </c>
+      <c r="I32" s="8" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="70" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B33" s="54" t="s">
+        <v>16</v>
+      </c>
+      <c r="C33" s="54" t="s">
+        <v>14</v>
+      </c>
+      <c r="D33" s="54" t="s">
+        <v>233</v>
+      </c>
+      <c r="E33" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="F33" s="54" t="n">
+        <v>1260</v>
+      </c>
+      <c r="G33" s="70" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H33" s="54" t="s">
+        <v>233</v>
+      </c>
+      <c r="I33" s="8" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="70" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B34" s="54" t="s">
+        <v>16</v>
+      </c>
+      <c r="C34" s="54" t="s">
+        <v>14</v>
+      </c>
+      <c r="D34" s="54" t="s">
+        <v>233</v>
+      </c>
+      <c r="E34" s="8" t="s">
+        <v>347</v>
+      </c>
+      <c r="F34" s="54" t="n">
+        <v>180</v>
+      </c>
+      <c r="G34" s="70" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H34" s="54" t="s">
+        <v>233</v>
+      </c>
+      <c r="I34" s="8" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="70" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B35" s="54" t="s">
+        <v>16</v>
+      </c>
+      <c r="C35" s="54" t="s">
+        <v>14</v>
+      </c>
+      <c r="D35" s="54" t="s">
+        <v>233</v>
+      </c>
+      <c r="E35" s="8" t="s">
+        <v>349</v>
+      </c>
+      <c r="F35" s="54" t="n">
+        <v>315</v>
+      </c>
+      <c r="G35" s="70" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H35" s="54" t="s">
+        <v>233</v>
+      </c>
+      <c r="I35" s="8" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="70" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B36" s="54" t="s">
+        <v>16</v>
+      </c>
+      <c r="C36" s="54" t="s">
+        <v>14</v>
+      </c>
+      <c r="D36" s="54" t="s">
+        <v>233</v>
+      </c>
+      <c r="E36" s="8" t="s">
+        <v>351</v>
+      </c>
+      <c r="F36" s="54" t="n">
+        <v>360</v>
+      </c>
+      <c r="G36" s="70" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H36" s="54" t="s">
+        <v>233</v>
+      </c>
+      <c r="I36" s="8" t="s">
+        <v>352</v>
       </c>
     </row>
   </sheetData>
@@ -5067,47 +5377,47 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>335</v>
+        <v>353</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>336</v>
+        <v>354</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>337</v>
+        <v>355</v>
       </c>
       <c r="B4" s="71" t="n">
         <v>1360</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>338</v>
+        <v>356</v>
       </c>
       <c r="D4" s="72" t="n">
         <f aca="false">B4-SUM(E8:E40)</f>
-        <v>190</v>
+        <v>-140</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>339</v>
+        <v>357</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>340</v>
+        <v>358</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>341</v>
+        <v>359</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>342</v>
+        <v>360</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>343</v>
+        <v>361</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>344</v>
+        <v>362</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5115,13 +5425,13 @@
         <v>46244</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>345</v>
+        <v>363</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>346</v>
+        <v>364</v>
       </c>
       <c r="E8" s="18" t="n">
         <v>344.16</v>
@@ -5136,13 +5446,13 @@
         <v>46245</v>
       </c>
       <c r="B9" s="68" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="C9" s="68" t="s">
-        <v>347</v>
+        <v>365</v>
       </c>
       <c r="D9" s="68" t="s">
-        <v>348</v>
+        <v>366</v>
       </c>
       <c r="E9" s="69" t="n">
         <v>-344.16</v>
@@ -5157,13 +5467,13 @@
         <v>46245</v>
       </c>
       <c r="B10" s="68" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="C10" s="68" t="s">
-        <v>349</v>
+        <v>367</v>
       </c>
       <c r="D10" s="68" t="s">
-        <v>346</v>
+        <v>364</v>
       </c>
       <c r="E10" s="69" t="n">
         <v>390</v>
@@ -5178,13 +5488,13 @@
         <v>46246</v>
       </c>
       <c r="B11" s="68" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="C11" s="68" t="s">
-        <v>350</v>
+        <v>368</v>
       </c>
       <c r="D11" s="68" t="s">
-        <v>346</v>
+        <v>364</v>
       </c>
       <c r="E11" s="69" t="n">
         <v>390</v>
@@ -5196,23 +5506,23 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="66" t="n">
-        <v>46273</v>
+        <v>46276</v>
       </c>
       <c r="B12" s="68" t="s">
-        <v>351</v>
+        <v>231</v>
       </c>
       <c r="C12" s="68" t="s">
-        <v>352</v>
+        <v>369</v>
       </c>
       <c r="D12" s="67" t="s">
-        <v>353</v>
+        <v>370</v>
       </c>
       <c r="E12" s="69" t="n">
-        <v>350</v>
+        <v>680</v>
       </c>
       <c r="F12" s="10" t="n">
         <f aca="false">IF(E12="","",$B$4-SUM($E$8:E12))</f>
-        <v>230</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5223,7 +5533,7 @@
         <v>14</v>
       </c>
       <c r="C13" s="68" t="s">
-        <v>354</v>
+        <v>371</v>
       </c>
       <c r="D13" s="67" t="s">
         <v>29</v>
@@ -5233,7 +5543,7 @@
       </c>
       <c r="F13" s="10" t="n">
         <f aca="false">IF(E13="","",$B$4-SUM($E$8:E13))</f>
-        <v>190</v>
+        <v>-140</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5397,23 +5707,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>355</v>
+        <v>372</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>356</v>
+        <v>373</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>337</v>
+        <v>355</v>
       </c>
       <c r="B4" s="71" t="n">
         <v>1130</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>338</v>
+        <v>356</v>
       </c>
       <c r="D4" s="72" t="n">
         <f aca="false">B4-SUM(E8:E40)</f>
@@ -5422,22 +5732,22 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>339</v>
+        <v>357</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>357</v>
+        <v>374</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>358</v>
+        <v>375</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>342</v>
+        <v>360</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>343</v>
+        <v>361</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>344</v>
+        <v>362</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5445,13 +5755,13 @@
         <v>46223</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>359</v>
+        <v>376</v>
       </c>
       <c r="D8" s="54" t="s">
-        <v>360</v>
+        <v>377</v>
       </c>
       <c r="E8" s="18" t="n">
         <v>311.98</v>
@@ -5466,13 +5776,13 @@
         <v>46225</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>361</v>
+        <v>378</v>
       </c>
       <c r="D9" s="54" t="s">
-        <v>362</v>
+        <v>379</v>
       </c>
       <c r="E9" s="18" t="n">
         <v>162.96</v>
@@ -5487,13 +5797,13 @@
         <v>46238</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>363</v>
+        <v>380</v>
       </c>
       <c r="D10" s="54" t="s">
-        <v>364</v>
+        <v>381</v>
       </c>
       <c r="E10" s="18" t="n">
         <v>148.53</v>
@@ -5508,13 +5818,13 @@
         <v>46250</v>
       </c>
       <c r="B11" s="67" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="C11" s="68" t="s">
-        <v>365</v>
+        <v>382</v>
       </c>
       <c r="D11" s="68" t="s">
-        <v>366</v>
+        <v>383</v>
       </c>
       <c r="E11" s="69" t="n">
         <v>47.99</v>
@@ -5532,10 +5842,10 @@
         <v>214</v>
       </c>
       <c r="C12" s="68" t="s">
-        <v>367</v>
+        <v>384</v>
       </c>
       <c r="D12" s="67" t="s">
-        <v>368</v>
+        <v>385</v>
       </c>
       <c r="E12" s="69" t="n">
         <v>481.26</v>
@@ -5561,13 +5871,13 @@
         <v>46244</v>
       </c>
       <c r="B14" s="68" t="s">
-        <v>369</v>
+        <v>386</v>
       </c>
       <c r="C14" s="68" t="s">
-        <v>370</v>
+        <v>387</v>
       </c>
       <c r="D14" s="67" t="s">
-        <v>368</v>
+        <v>385</v>
       </c>
       <c r="E14" s="69" t="n">
         <v>40.18</v>
@@ -5725,44 +6035,44 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>371</v>
+        <v>388</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>372</v>
+        <v>389</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>373</v>
+        <v>390</v>
       </c>
       <c r="B4" s="71" t="n">
         <v>5000</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>338</v>
+        <v>356</v>
       </c>
       <c r="D4" s="72" t="n">
         <f aca="false">B4-SUM(D8:D40)</f>
-        <v>4377.36</v>
+        <v>2262.36</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>339</v>
+        <v>357</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>374</v>
+        <v>391</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>375</v>
+        <v>392</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>343</v>
+        <v>361</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>344</v>
+        <v>362</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5770,10 +6080,10 @@
         <v>46248</v>
       </c>
       <c r="B8" s="68" t="s">
-        <v>376</v>
+        <v>393</v>
       </c>
       <c r="C8" s="68" t="s">
-        <v>377</v>
+        <v>394</v>
       </c>
       <c r="D8" s="69" t="n">
         <v>250</v>
@@ -5788,7 +6098,7 @@
         <v>46251</v>
       </c>
       <c r="B9" s="68" t="s">
-        <v>378</v>
+        <v>395</v>
       </c>
       <c r="C9" s="68" t="s">
         <v>214</v>
@@ -5806,10 +6116,10 @@
         <v>46251</v>
       </c>
       <c r="B10" s="68" t="s">
-        <v>379</v>
+        <v>396</v>
       </c>
       <c r="C10" s="68" t="s">
-        <v>380</v>
+        <v>397</v>
       </c>
       <c r="D10" s="69" t="n">
         <v>62.9</v>
@@ -5824,10 +6134,10 @@
         <v>46258</v>
       </c>
       <c r="B11" s="68" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
       <c r="C11" s="68" t="s">
-        <v>381</v>
+        <v>398</v>
       </c>
       <c r="D11" s="69" t="n">
         <v>141.66</v>
@@ -5842,7 +6152,7 @@
         <v>46275</v>
       </c>
       <c r="B12" s="68" t="s">
-        <v>382</v>
+        <v>399</v>
       </c>
       <c r="C12" s="68" t="s">
         <v>11</v>
@@ -5856,43 +6166,75 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="73"/>
-      <c r="B13" s="74"/>
-      <c r="C13" s="74"/>
-      <c r="D13" s="75"/>
-      <c r="E13" s="10" t="str">
+      <c r="A13" s="66" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B13" s="68" t="s">
+        <v>345</v>
+      </c>
+      <c r="C13" s="68" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="69" t="n">
+        <v>1260</v>
+      </c>
+      <c r="E13" s="10" t="n">
         <f aca="false">IF(D13="","",$B$4-SUM($D$8:D13))</f>
-        <v/>
+        <v>3117.36</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="73"/>
-      <c r="B14" s="74"/>
-      <c r="C14" s="74"/>
-      <c r="D14" s="75"/>
-      <c r="E14" s="10" t="str">
+      <c r="A14" s="66" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B14" s="68" t="s">
+        <v>400</v>
+      </c>
+      <c r="C14" s="68" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" s="69" t="n">
+        <v>180</v>
+      </c>
+      <c r="E14" s="10" t="n">
         <f aca="false">IF(D14="","",$B$4-SUM($D$8:D14))</f>
-        <v/>
+        <v>2937.36</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="73"/>
-      <c r="B15" s="74"/>
-      <c r="C15" s="74"/>
-      <c r="D15" s="75"/>
-      <c r="E15" s="10" t="str">
+      <c r="A15" s="66" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B15" s="68" t="s">
+        <v>401</v>
+      </c>
+      <c r="C15" s="68" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="69" t="n">
+        <v>315</v>
+      </c>
+      <c r="E15" s="10" t="n">
         <f aca="false">IF(D15="","",$B$4-SUM($D$8:D15))</f>
-        <v/>
+        <v>2622.36</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="73"/>
-      <c r="B16" s="74"/>
-      <c r="C16" s="74"/>
-      <c r="D16" s="75"/>
-      <c r="E16" s="10" t="str">
+      <c r="A16" s="66" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B16" s="68" t="s">
+        <v>351</v>
+      </c>
+      <c r="C16" s="68" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="69" t="n">
+        <v>360</v>
+      </c>
+      <c r="E16" s="10" t="n">
         <f aca="false">IF(D16="","",$B$4-SUM($D$8:D16))</f>
-        <v/>
+        <v>2262.36</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>